<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-02-07 13:39:28
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_B2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_B2_session_analysis.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>77.6%</t>
+          <t>78.6%</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>72.5%</t>
+          <t>72.2%</t>
         </is>
       </c>
     </row>
@@ -1598,22 +1598,22 @@
         <v>40</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q19" s="4" t="n">
         <v>4</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>82.5%</t>
         </is>
       </c>
       <c r="S19" s="4" t="inlineStr">
         <is>
-          <t>71.3%</t>
+          <t>71.5%</t>
         </is>
       </c>
     </row>
@@ -1676,22 +1676,22 @@
         <v>42</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Q20" s="4" t="n">
         <v>4</v>
       </c>
       <c r="R20" s="4" t="inlineStr">
         <is>
-          <t>71.4%</t>
+          <t>73.8%</t>
         </is>
       </c>
       <c r="S20" s="4" t="inlineStr">
         <is>
-          <t>77.8%</t>
+          <t>75.4%</t>
         </is>
       </c>
     </row>
@@ -1832,17 +1832,17 @@
         <v>40</v>
       </c>
       <c r="O22" s="4" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q22" s="4" t="n">
         <v>4</v>
       </c>
       <c r="R22" s="4" t="inlineStr">
         <is>
-          <t>82.5%</t>
+          <t>85.0%</t>
         </is>
       </c>
       <c r="S22" s="4" t="inlineStr">
@@ -8539,45 +8539,45 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="5" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B177" s="5" t="inlineStr">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B177" s="2" t="inlineStr">
         <is>
           <t>B2-C1</t>
         </is>
       </c>
-      <c r="C177" s="5" t="inlineStr">
+      <c r="C177" s="2" t="inlineStr">
         <is>
           <t>GASTROENTEROLOGY</t>
         </is>
       </c>
-      <c r="D177" s="5" t="inlineStr">
+      <c r="D177" s="2" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E177" s="5" t="inlineStr">
+      <c r="E177" s="2" t="inlineStr">
         <is>
           <t>07/02/2026</t>
         </is>
       </c>
-      <c r="F177" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G177" s="5" t="inlineStr"/>
-      <c r="H177" s="5" t="inlineStr">
-        <is>
-          <t>0/52</t>
-        </is>
-      </c>
-      <c r="I177" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F177" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G177" s="2" t="inlineStr"/>
+      <c r="H177" s="2" t="inlineStr">
+        <is>
+          <t>40/52</t>
+        </is>
+      </c>
+      <c r="I177" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -10259,45 +10259,45 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="5" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B217" s="5" t="inlineStr">
+      <c r="A217" s="2" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B217" s="2" t="inlineStr">
         <is>
           <t>B2-C2</t>
         </is>
       </c>
-      <c r="C217" s="5" t="inlineStr">
+      <c r="C217" s="2" t="inlineStr">
         <is>
           <t>GASTROENTEROLOGY</t>
         </is>
       </c>
-      <c r="D217" s="5" t="inlineStr">
+      <c r="D217" s="2" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E217" s="5" t="inlineStr">
+      <c r="E217" s="2" t="inlineStr">
         <is>
           <t>07/02/2026</t>
         </is>
       </c>
-      <c r="F217" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G217" s="5" t="inlineStr"/>
-      <c r="H217" s="5" t="inlineStr">
-        <is>
-          <t>0/51</t>
-        </is>
-      </c>
-      <c r="I217" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F217" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G217" s="2" t="inlineStr"/>
+      <c r="H217" s="2" t="inlineStr">
+        <is>
+          <t>2/51</t>
+        </is>
+      </c>
+      <c r="I217" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -14645,45 +14645,45 @@
       </c>
     </row>
     <row r="319">
-      <c r="A319" s="5" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B319" s="5" t="inlineStr">
+      <c r="A319" s="2" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B319" s="2" t="inlineStr">
         <is>
           <t>B2-D2</t>
         </is>
       </c>
-      <c r="C319" s="5" t="inlineStr">
+      <c r="C319" s="2" t="inlineStr">
         <is>
           <t>RHEUMATOLOGY</t>
         </is>
       </c>
-      <c r="D319" s="5" t="inlineStr">
+      <c r="D319" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E319" s="5" t="inlineStr">
+      <c r="E319" s="2" t="inlineStr">
         <is>
           <t>07/02/2026</t>
         </is>
       </c>
-      <c r="F319" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G319" s="5" t="inlineStr"/>
-      <c r="H319" s="5" t="inlineStr">
-        <is>
-          <t>0/61</t>
-        </is>
-      </c>
-      <c r="I319" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F319" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G319" s="2" t="inlineStr"/>
+      <c r="H319" s="2" t="inlineStr">
+        <is>
+          <t>34/61</t>
+        </is>
+      </c>
+      <c r="I319" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-02-08 14:22:23
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_B2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_B2_session_analysis.xlsx
@@ -1769,7 +1769,7 @@
       </c>
       <c r="S21" s="4" t="inlineStr">
         <is>
-          <t>70.4%</t>
+          <t>70.6%</t>
         </is>
       </c>
     </row>
@@ -12376,7 +12376,7 @@
       </c>
       <c r="H265" s="2" t="inlineStr">
         <is>
-          <t>14/28</t>
+          <t>15/28</t>
         </is>
       </c>
       <c r="I265" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-02-08 21:21:18
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_B2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_B2_session_analysis.xlsx
@@ -2190,7 +2190,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>160715@med.asu.edu.eg</t>
+        </is>
+      </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
           <t>25/25</t>
@@ -3929,7 +3933,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G69" s="2" t="inlineStr"/>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>160715@med.asu.edu.eg</t>
+        </is>
+      </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
           <t>18/23</t>

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-02-09 09:56:45
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_B2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_B2_session_analysis.xlsx
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>80.4%</t>
+          <t>80.7%</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>72.1%</t>
+          <t>71.9%</t>
         </is>
       </c>
     </row>
@@ -1832,22 +1832,22 @@
         <v>40</v>
       </c>
       <c r="O22" s="4" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q22" s="4" t="n">
         <v>2</v>
       </c>
       <c r="R22" s="4" t="inlineStr">
         <is>
-          <t>87.5%</t>
+          <t>90.0%</t>
         </is>
       </c>
       <c r="S22" s="4" t="inlineStr">
         <is>
-          <t>56.4%</t>
+          <t>55.4%</t>
         </is>
       </c>
     </row>
@@ -14759,45 +14759,45 @@
       </c>
     </row>
     <row r="321">
-      <c r="A321" s="5" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B321" s="5" t="inlineStr">
+      <c r="A321" s="2" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B321" s="2" t="inlineStr">
         <is>
           <t>B2-D2</t>
         </is>
       </c>
-      <c r="C321" s="5" t="inlineStr">
+      <c r="C321" s="2" t="inlineStr">
         <is>
           <t>RHEUMATOLOGY</t>
         </is>
       </c>
-      <c r="D321" s="5" t="inlineStr">
+      <c r="D321" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E321" s="5" t="inlineStr">
+      <c r="E321" s="2" t="inlineStr">
         <is>
           <t>09/02/2026</t>
         </is>
       </c>
-      <c r="F321" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G321" s="5" t="inlineStr"/>
-      <c r="H321" s="5" t="inlineStr">
-        <is>
-          <t>0/61</t>
-        </is>
-      </c>
-      <c r="I321" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F321" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G321" s="2" t="inlineStr"/>
+      <c r="H321" s="2" t="inlineStr">
+        <is>
+          <t>11/61</t>
+        </is>
+      </c>
+      <c r="I321" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-02-11 12:56:44
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_B2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_B2_session_analysis.xlsx
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="7">
@@ -842,7 +842,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8">
@@ -945,7 +945,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>85.1%</t>
+          <t>85.4%</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>71.5%</t>
+          <t>71.4%</t>
         </is>
       </c>
     </row>
@@ -1829,22 +1829,22 @@
         <v>40</v>
       </c>
       <c r="O22" s="4" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q22" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R22" s="4" t="inlineStr">
         <is>
-          <t>92.5%</t>
+          <t>95.0%</t>
         </is>
       </c>
       <c r="S22" s="4" t="inlineStr">
         <is>
-          <t>55.1%</t>
+          <t>55.2%</t>
         </is>
       </c>
     </row>
@@ -14918,45 +14918,45 @@
       </c>
     </row>
     <row r="323">
-      <c r="A323" s="5" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B323" s="5" t="inlineStr">
+      <c r="A323" s="2" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B323" s="2" t="inlineStr">
         <is>
           <t>B2-D2</t>
         </is>
       </c>
-      <c r="C323" s="5" t="inlineStr">
+      <c r="C323" s="2" t="inlineStr">
         <is>
           <t>RHEUMATOLOGY</t>
         </is>
       </c>
-      <c r="D323" s="5" t="inlineStr">
+      <c r="D323" s="2" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E323" s="5" t="inlineStr">
+      <c r="E323" s="2" t="inlineStr">
         <is>
           <t>11/02/2026</t>
         </is>
       </c>
-      <c r="F323" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G323" s="5" t="inlineStr"/>
-      <c r="H323" s="5" t="inlineStr">
-        <is>
-          <t>0/61</t>
-        </is>
-      </c>
-      <c r="I323" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F323" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G323" s="2" t="inlineStr"/>
+      <c r="H323" s="2" t="inlineStr">
+        <is>
+          <t>35/61</t>
+        </is>
+      </c>
+      <c r="I323" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-02-11 17:00:38
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_B2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_B2_session_analysis.xlsx
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>275</v>
+        <v>277</v>
       </c>
     </row>
     <row r="7">
@@ -842,7 +842,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8">
@@ -945,7 +945,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>85.4%</t>
+          <t>86.0%</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>71.4%</t>
+          <t>71.5%</t>
         </is>
       </c>
     </row>
@@ -1595,17 +1595,17 @@
         <v>40</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q19" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>85.0%</t>
+          <t>87.5%</t>
         </is>
       </c>
       <c r="S19" s="4" t="inlineStr">
@@ -1673,22 +1673,22 @@
         <v>42</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="P20" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q20" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R20" s="4" t="inlineStr">
         <is>
-          <t>78.6%</t>
+          <t>81.0%</t>
         </is>
       </c>
       <c r="S20" s="4" t="inlineStr">
         <is>
-          <t>73.4%</t>
+          <t>74.0%</t>
         </is>
       </c>
     </row>
@@ -8749,45 +8749,49 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="5" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B180" s="5" t="inlineStr">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
         <is>
           <t>B2-C1</t>
         </is>
       </c>
-      <c r="C180" s="5" t="inlineStr">
+      <c r="C180" s="2" t="inlineStr">
         <is>
           <t>GASTROENTEROLOGY</t>
         </is>
       </c>
-      <c r="D180" s="5" t="inlineStr">
+      <c r="D180" s="2" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="E180" s="5" t="inlineStr">
+      <c r="E180" s="2" t="inlineStr">
         <is>
           <t>10/02/2026</t>
         </is>
       </c>
-      <c r="F180" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G180" s="5" t="inlineStr"/>
-      <c r="H180" s="5" t="inlineStr">
-        <is>
-          <t>0/52</t>
-        </is>
-      </c>
-      <c r="I180" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F180" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G180" s="2" t="inlineStr">
+        <is>
+          <t>emp17066@med.asu.edu.eg</t>
+        </is>
+      </c>
+      <c r="H180" s="2" t="inlineStr">
+        <is>
+          <t>37/52</t>
+        </is>
+      </c>
+      <c r="I180" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -10168,45 +10172,49 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="5" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B213" s="5" t="inlineStr">
+      <c r="A213" s="2" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B213" s="2" t="inlineStr">
         <is>
           <t>B2-C2</t>
         </is>
       </c>
-      <c r="C213" s="5" t="inlineStr">
+      <c r="C213" s="2" t="inlineStr">
         <is>
           <t>GASTROENTEROLOGY</t>
         </is>
       </c>
-      <c r="D213" s="5" t="inlineStr">
+      <c r="D213" s="2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E213" s="5" t="inlineStr">
+      <c r="E213" s="2" t="inlineStr">
         <is>
           <t>18/01/2026</t>
         </is>
       </c>
-      <c r="F213" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G213" s="5" t="inlineStr"/>
-      <c r="H213" s="5" t="inlineStr">
-        <is>
-          <t>0/51</t>
-        </is>
-      </c>
-      <c r="I213" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F213" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G213" s="2" t="inlineStr">
+        <is>
+          <t>emp17066@med.asu.edu.eg</t>
+        </is>
+      </c>
+      <c r="H213" s="2" t="inlineStr">
+        <is>
+          <t>48/51</t>
+        </is>
+      </c>
+      <c r="I213" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-02-11 18:54:48
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_B2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_B2_session_analysis.xlsx
@@ -571,7 +571,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
           <t>18/25</t>
@@ -619,7 +623,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
           <t>20/25</t>
@@ -672,7 +680,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
           <t>20/25</t>
@@ -723,7 +735,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
           <t>18/25</t>
@@ -774,7 +790,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
           <t>22/25</t>
@@ -791,7 +811,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>277</v>
+        <v>280</v>
       </c>
     </row>
     <row r="7">
@@ -825,7 +845,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
           <t>22/25</t>
@@ -842,7 +866,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8">
@@ -876,7 +900,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
           <t>23/25</t>
@@ -927,7 +955,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
           <t>21/25</t>
@@ -945,7 +977,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>86.0%</t>
+          <t>87.0%</t>
         </is>
       </c>
     </row>
@@ -980,7 +1012,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
           <t>22/25</t>
@@ -998,7 +1034,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>71.5%</t>
+          <t>71.3%</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1069,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
           <t>18/25</t>
@@ -1439,22 +1479,22 @@
         <v>40</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q17" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>92.5%</t>
+          <t>95.0%</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>71.4%</t>
+          <t>70.5%</t>
         </is>
       </c>
     </row>
@@ -1517,22 +1557,22 @@
         <v>40</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>82.5%</t>
+          <t>85.0%</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>70.3%</t>
+          <t>70.4%</t>
         </is>
       </c>
     </row>
@@ -1751,22 +1791,22 @@
         <v>40</v>
       </c>
       <c r="O21" s="4" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P21" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q21" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R21" s="4" t="inlineStr">
         <is>
-          <t>77.5%</t>
+          <t>80.0%</t>
         </is>
       </c>
       <c r="S21" s="4" t="inlineStr">
         <is>
-          <t>69.4%</t>
+          <t>68.6%</t>
         </is>
       </c>
     </row>
@@ -2781,7 +2821,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr"/>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
           <t>17/23</t>
@@ -2824,7 +2868,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G43" s="2" t="inlineStr"/>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
           <t>22/23</t>
@@ -2867,7 +2915,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr"/>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
           <t>22/23</t>
@@ -2910,7 +2962,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G45" s="2" t="inlineStr"/>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
           <t>19/23</t>
@@ -2953,7 +3009,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr"/>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
           <t>21/23</t>
@@ -2996,7 +3056,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G47" s="2" t="inlineStr"/>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
           <t>19/23</t>
@@ -3039,7 +3103,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G48" s="2" t="inlineStr"/>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
           <t>21/23</t>
@@ -3082,7 +3150,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G49" s="2" t="inlineStr"/>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
           <t>23/23</t>
@@ -3125,7 +3197,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G50" s="2" t="inlineStr"/>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
           <t>21/23</t>
@@ -3168,7 +3244,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G51" s="2" t="inlineStr"/>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
           <t>19/23</t>
@@ -4736,7 +4816,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G87" s="2" t="inlineStr"/>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
           <t>15/40</t>
@@ -4878,45 +4962,45 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="5" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B91" s="5" t="inlineStr">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
         <is>
           <t>B2-B1</t>
         </is>
       </c>
-      <c r="C91" s="5" t="inlineStr">
+      <c r="C91" s="2" t="inlineStr">
         <is>
           <t>ENDOCRINOLOGY</t>
         </is>
       </c>
-      <c r="D91" s="5" t="inlineStr">
+      <c r="D91" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E91" s="5" t="inlineStr">
+      <c r="E91" s="2" t="inlineStr">
         <is>
           <t>11/02/2026</t>
         </is>
       </c>
-      <c r="F91" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G91" s="5" t="inlineStr"/>
-      <c r="H91" s="5" t="inlineStr">
-        <is>
-          <t>0/40</t>
-        </is>
-      </c>
-      <c r="I91" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr"/>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>16/40</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -6476,7 +6560,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G127" s="2" t="inlineStr"/>
+      <c r="G127" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H127" s="2" t="inlineStr">
         <is>
           <t>20/35</t>
@@ -6618,45 +6706,45 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="5" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B131" s="5" t="inlineStr">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
         <is>
           <t>B2-B2</t>
         </is>
       </c>
-      <c r="C131" s="5" t="inlineStr">
+      <c r="C131" s="2" t="inlineStr">
         <is>
           <t>ENDOCRINOLOGY</t>
         </is>
       </c>
-      <c r="D131" s="5" t="inlineStr">
+      <c r="D131" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E131" s="5" t="inlineStr">
+      <c r="E131" s="2" t="inlineStr">
         <is>
           <t>11/02/2026</t>
         </is>
       </c>
-      <c r="F131" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G131" s="5" t="inlineStr"/>
-      <c r="H131" s="5" t="inlineStr">
-        <is>
-          <t>0/35</t>
-        </is>
-      </c>
-      <c r="I131" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F131" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G131" s="2" t="inlineStr"/>
+      <c r="H131" s="2" t="inlineStr">
+        <is>
+          <t>26/35</t>
+        </is>
+      </c>
+      <c r="I131" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -8001,7 +8089,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G162" s="2" t="inlineStr"/>
+      <c r="G162" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H162" s="2" t="inlineStr">
         <is>
           <t>45/52</t>
@@ -8044,7 +8136,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G163" s="2" t="inlineStr"/>
+      <c r="G163" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H163" s="2" t="inlineStr">
         <is>
           <t>43/52</t>
@@ -8087,7 +8183,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G164" s="2" t="inlineStr"/>
+      <c r="G164" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H164" s="2" t="inlineStr">
         <is>
           <t>51/52</t>
@@ -8130,7 +8230,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G165" s="2" t="inlineStr"/>
+      <c r="G165" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H165" s="2" t="inlineStr">
         <is>
           <t>46/52</t>
@@ -8216,7 +8320,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G167" s="2" t="inlineStr"/>
+      <c r="G167" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H167" s="2" t="inlineStr">
         <is>
           <t>33/52</t>
@@ -8259,7 +8367,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G168" s="2" t="inlineStr"/>
+      <c r="G168" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H168" s="2" t="inlineStr">
         <is>
           <t>48/52</t>
@@ -8302,7 +8414,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G169" s="2" t="inlineStr"/>
+      <c r="G169" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H169" s="2" t="inlineStr">
         <is>
           <t>46/52</t>
@@ -8345,7 +8461,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G170" s="2" t="inlineStr"/>
+      <c r="G170" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
           <t>51/52</t>
@@ -8388,7 +8508,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G171" s="2" t="inlineStr"/>
+      <c r="G171" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H171" s="2" t="inlineStr">
         <is>
           <t>47/52</t>
@@ -9729,7 +9853,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G202" s="2" t="inlineStr"/>
+      <c r="G202" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H202" s="2" t="inlineStr">
         <is>
           <t>44/51</t>
@@ -9772,7 +9900,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G203" s="2" t="inlineStr"/>
+      <c r="G203" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H203" s="2" t="inlineStr">
         <is>
           <t>41/51</t>
@@ -9815,7 +9947,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G204" s="2" t="inlineStr"/>
+      <c r="G204" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H204" s="2" t="inlineStr">
         <is>
           <t>49/51</t>
@@ -9858,7 +9994,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G205" s="2" t="inlineStr"/>
+      <c r="G205" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H205" s="2" t="inlineStr">
         <is>
           <t>47/51</t>
@@ -9944,7 +10084,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G207" s="2" t="inlineStr"/>
+      <c r="G207" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H207" s="2" t="inlineStr">
         <is>
           <t>34/51</t>
@@ -9987,7 +10131,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G208" s="2" t="inlineStr"/>
+      <c r="G208" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H208" s="2" t="inlineStr">
         <is>
           <t>48/51</t>
@@ -10030,7 +10178,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G209" s="2" t="inlineStr"/>
+      <c r="G209" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H209" s="2" t="inlineStr">
         <is>
           <t>46/51</t>
@@ -10073,7 +10225,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G210" s="2" t="inlineStr"/>
+      <c r="G210" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H210" s="2" t="inlineStr">
         <is>
           <t>43/51</t>
@@ -10116,7 +10272,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G211" s="2" t="inlineStr"/>
+      <c r="G211" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H211" s="2" t="inlineStr">
         <is>
           <t>47/51</t>
@@ -11547,7 +11707,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G244" s="2" t="inlineStr"/>
+      <c r="G244" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H244" s="2" t="inlineStr">
         <is>
           <t>26/28</t>
@@ -11590,7 +11754,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G245" s="2" t="inlineStr"/>
+      <c r="G245" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H245" s="2" t="inlineStr">
         <is>
           <t>20/28</t>
@@ -11633,7 +11801,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G246" s="2" t="inlineStr"/>
+      <c r="G246" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H246" s="2" t="inlineStr">
         <is>
           <t>26/28</t>
@@ -11676,7 +11848,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G247" s="2" t="inlineStr"/>
+      <c r="G247" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H247" s="2" t="inlineStr">
         <is>
           <t>25/28</t>
@@ -11719,7 +11895,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G248" s="2" t="inlineStr"/>
+      <c r="G248" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H248" s="2" t="inlineStr">
         <is>
           <t>27/28</t>
@@ -11762,7 +11942,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G249" s="2" t="inlineStr"/>
+      <c r="G249" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H249" s="2" t="inlineStr">
         <is>
           <t>22/28</t>
@@ -11805,7 +11989,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G250" s="2" t="inlineStr"/>
+      <c r="G250" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H250" s="2" t="inlineStr">
         <is>
           <t>26/28</t>
@@ -11848,7 +12036,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G251" s="2" t="inlineStr"/>
+      <c r="G251" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H251" s="2" t="inlineStr">
         <is>
           <t>25/28</t>
@@ -11891,7 +12083,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G252" s="2" t="inlineStr"/>
+      <c r="G252" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H252" s="2" t="inlineStr">
         <is>
           <t>26/28</t>
@@ -11934,7 +12130,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G253" s="2" t="inlineStr"/>
+      <c r="G253" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H253" s="2" t="inlineStr">
         <is>
           <t>24/28</t>
@@ -12281,7 +12481,7 @@
       <c r="G261" s="2" t="inlineStr"/>
       <c r="H261" s="2" t="inlineStr">
         <is>
-          <t>1/28</t>
+          <t>4/28</t>
         </is>
       </c>
       <c r="I261" s="2" t="inlineStr">
@@ -12291,45 +12491,45 @@
       </c>
     </row>
     <row r="262">
-      <c r="A262" s="5" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B262" s="5" t="inlineStr">
+      <c r="A262" s="2" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B262" s="2" t="inlineStr">
         <is>
           <t>B2-D1</t>
         </is>
       </c>
-      <c r="C262" s="5" t="inlineStr">
+      <c r="C262" s="2" t="inlineStr">
         <is>
           <t>GASTROENTEROLOGY</t>
         </is>
       </c>
-      <c r="D262" s="5" t="inlineStr">
+      <c r="D262" s="2" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="E262" s="5" t="inlineStr">
+      <c r="E262" s="2" t="inlineStr">
         <is>
           <t>13/01/2026</t>
         </is>
       </c>
-      <c r="F262" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G262" s="5" t="inlineStr"/>
-      <c r="H262" s="5" t="inlineStr">
-        <is>
-          <t>0/28</t>
-        </is>
-      </c>
-      <c r="I262" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F262" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G262" s="2" t="inlineStr"/>
+      <c r="H262" s="2" t="inlineStr">
+        <is>
+          <t>10/28</t>
+        </is>
+      </c>
+      <c r="I262" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -13279,7 +13479,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G284" s="2" t="inlineStr"/>
+      <c r="G284" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H284" s="2" t="inlineStr">
         <is>
           <t>40/61</t>
@@ -13322,7 +13526,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G285" s="2" t="inlineStr"/>
+      <c r="G285" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H285" s="2" t="inlineStr">
         <is>
           <t>41/61</t>
@@ -13365,7 +13573,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G286" s="2" t="inlineStr"/>
+      <c r="G286" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H286" s="2" t="inlineStr">
         <is>
           <t>42/61</t>
@@ -13408,7 +13620,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G287" s="2" t="inlineStr"/>
+      <c r="G287" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H287" s="2" t="inlineStr">
         <is>
           <t>39/61</t>
@@ -13451,7 +13667,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G288" s="2" t="inlineStr"/>
+      <c r="G288" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H288" s="2" t="inlineStr">
         <is>
           <t>40/61</t>
@@ -13494,7 +13714,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G289" s="2" t="inlineStr"/>
+      <c r="G289" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H289" s="2" t="inlineStr">
         <is>
           <t>33/61</t>
@@ -13537,7 +13761,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G290" s="2" t="inlineStr"/>
+      <c r="G290" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H290" s="2" t="inlineStr">
         <is>
           <t>36/61</t>
@@ -13580,7 +13808,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G291" s="2" t="inlineStr"/>
+      <c r="G291" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H291" s="2" t="inlineStr">
         <is>
           <t>45/61</t>
@@ -13623,7 +13855,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G292" s="2" t="inlineStr"/>
+      <c r="G292" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H292" s="2" t="inlineStr">
         <is>
           <t>42/61</t>
@@ -13666,7 +13902,11 @@
           <t>09:00:00</t>
         </is>
       </c>
-      <c r="G293" s="2" t="inlineStr"/>
+      <c r="G293" s="2" t="inlineStr">
+        <is>
+          <t>776626600547</t>
+        </is>
+      </c>
       <c r="H293" s="2" t="inlineStr">
         <is>
           <t>43/61</t>
@@ -14056,7 +14296,7 @@
       <c r="G302" s="2" t="inlineStr"/>
       <c r="H302" s="2" t="inlineStr">
         <is>
-          <t>40/61</t>
+          <t>41/61</t>
         </is>
       </c>
       <c r="I302" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sync attendance_reports, modules_schedules, and assets from main repo - 2026-02-12 11:36:03
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_B2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_B2_session_analysis.xlsx
@@ -811,7 +811,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="7">
@@ -866,7 +866,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8">
@@ -977,7 +977,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>87.6%</t>
+          <t>87.9%</t>
         </is>
       </c>
     </row>
@@ -1034,7 +1034,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>71.1%</t>
+          <t>71.2%</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>79.1%</t>
+          <t>79.7%</t>
         </is>
       </c>
     </row>
@@ -1401,22 +1401,22 @@
         <v>40</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q16" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>85.0%</t>
+          <t>87.5%</t>
         </is>
       </c>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>82.1%</t>
+          <t>82.4%</t>
         </is>
       </c>
     </row>
@@ -2543,7 +2543,7 @@
       <c r="G35" s="2" t="inlineStr"/>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>14/25</t>
+          <t>19/25</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -4306,45 +4306,45 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="5" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B75" s="5" t="inlineStr">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
         <is>
           <t>B2-A2</t>
         </is>
       </c>
-      <c r="C75" s="5" t="inlineStr">
+      <c r="C75" s="2" t="inlineStr">
         <is>
           <t>PHYSICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D75" s="5" t="inlineStr">
+      <c r="D75" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E75" s="5" t="inlineStr">
+      <c r="E75" s="2" t="inlineStr">
         <is>
           <t>21/01/2026</t>
         </is>
       </c>
-      <c r="F75" s="5" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G75" s="5" t="inlineStr"/>
-      <c r="H75" s="5" t="inlineStr">
-        <is>
-          <t>0/23</t>
-        </is>
-      </c>
-      <c r="I75" s="5" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr"/>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>21/23</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>